<commit_message>
New XLSL Sheet added
</commit_message>
<xml_diff>
--- a/Krishna Assignment.xlsx
+++ b/Krishna Assignment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5F10C37138A14469/Desktop/SAP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="688" documentId="8_{C4CB7184-34CC-4D88-B47A-A2840B42DD0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44740330-921F-489F-9DA2-325C4D79A2D2}"/>
+  <xr:revisionPtr revIDLastSave="694" documentId="8_{C4CB7184-34CC-4D88-B47A-A2840B42DD0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96ABB39C-CFB4-430C-B10A-41371D9B5D99}"/>
   <bookViews>
-    <workbookView xWindow="2976" yWindow="1488" windowWidth="17280" windowHeight="9420" xr2:uid="{26A7549B-DA9D-4851-B6BF-1D9C48768FDE}"/>
+    <workbookView xWindow="4020" yWindow="2532" windowWidth="17280" windowHeight="9420" xr2:uid="{26A7549B-DA9D-4851-B6BF-1D9C48768FDE}"/>
   </bookViews>
   <sheets>
     <sheet name="ABAP" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="386">
   <si>
     <t>Date</t>
   </si>
@@ -1281,12 +1281,36 @@
   <si>
     <t>Assignment 40</t>
   </si>
+  <si>
+    <t>Session Method</t>
+  </si>
+  <si>
+    <t>1.what is session method?</t>
+  </si>
+  <si>
+    <t>2.Why and when we go for call transaction and session method ?</t>
+  </si>
+  <si>
+    <t>3.Differnce between session method and call transaction method?</t>
+  </si>
+  <si>
+    <t>5.try to upload some record which is already created and upload using session method?</t>
+  </si>
+  <si>
+    <t>6.explore all 3 session method funtion module?</t>
+  </si>
+  <si>
+    <t>7.what is use of keep,dest,group,holdate in bdc_open_group?</t>
+  </si>
+  <si>
+    <t>4.what is advantage of session method over call transaction?</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="29" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1509,6 +1533,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -1549,7 +1581,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1643,6 +1675,7 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1956,9 +1989,36 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{D6E18F14-8040-4D8C-B947-4F786859EBD0}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;e2f7922a-27c5-4481-b965-cca2a582c21d&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{970B57CD-2E87-4C38-BB7E-7DC8579D2EE2}">
-  <dimension ref="A2:E390"/>
+  <dimension ref="A2:E400"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.6640625" customWidth="1"/>
@@ -3888,6 +3948,46 @@
     <row r="390" spans="2:2" ht="18" x14ac:dyDescent="0.35">
       <c r="B390" s="16" t="s">
         <v>376</v>
+      </c>
+    </row>
+    <row r="393" spans="2:2" ht="18" x14ac:dyDescent="0.35">
+      <c r="B393" s="45" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="394" spans="2:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B394" s="29" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="395" spans="2:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B395" s="29" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="396" spans="2:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B396" s="29" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="397" spans="2:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B397" s="29" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="398" spans="2:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B398" s="29" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="399" spans="2:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B399" s="29" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="400" spans="2:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B400" s="29" t="s">
+        <v>384</v>
       </c>
     </row>
   </sheetData>

</xml_diff>